<commit_message>
Adota base de curadoria manual como fonte oficial e re-roda todas as análises
- preparar_base.py: normaliza a curadoria manual para o schema canônico
  c4ai_publicacoes.xlsx (407 pubs; consolida AI HEALTH; corrige 2 grupos
  deslocados para AGRIBIO).
- analise_publicacoes e coword_analysis.py: passam a usar c4ai_publicacoes.xlsx
  como entrada padrão.
- Regenera Figuras 1-11, tabelas, relatório executivo e a co-word.
- Atualiza RELATORIO.md, documento_analise.tex e README.md com os números
  novos (407 pubs; pico 2023=189; KEML #2; HHI 1998; top-3 62,6%) e adiciona a
  seção de co-word ao .tex.
- Remove artefatos _manual redundantes.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Fvrdaa5i99DsPUToDczGGv
</commit_message>
<xml_diff>
--- a/output/c4ai_matriz_grupo_ano.xlsx
+++ b/output/c4ai_matriz_grupo_ano.xlsx
@@ -453,19 +453,19 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D2" t="n">
         <v>16</v>
       </c>
       <c r="E2" t="n">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G2" t="n">
-        <v>58</v>
+        <v>54</v>
       </c>
     </row>
     <row r="3">
@@ -509,13 +509,13 @@
         <v>23</v>
       </c>
       <c r="E4" t="n">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="F4" t="n">
         <v>3</v>
       </c>
       <c r="G4" t="n">
-        <v>53</v>
+        <v>50</v>
       </c>
     </row>
     <row r="5">
@@ -653,19 +653,19 @@
         <v>5</v>
       </c>
       <c r="C10" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D10" t="n">
         <v>103</v>
       </c>
       <c r="E10" t="n">
-        <v>199</v>
+        <v>189</v>
       </c>
       <c r="F10" t="n">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="G10" t="n">
-        <v>413</v>
+        <v>406</v>
       </c>
     </row>
   </sheetData>

</xml_diff>